<commit_message>
Fix nöbet_başı distribution to scale proportionally with seniority
</commit_message>
<xml_diff>
--- a/data/doctors_september2026.xlsx
+++ b/data/doctors_september2026.xlsx
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Dr. Ozan Sarıkaya</t>
+          <t>Dr. Test01</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -459,7 +459,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dr. Hasan Can Sağlam</t>
+          <t>Dr. Test02</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -477,7 +477,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dr. Alp Eren Aksoy</t>
+          <t>Dr. Test03</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -495,7 +495,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dr. Asena Karabacak</t>
+          <t>Dr. Test04</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -513,7 +513,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dr. Aslı Nur Kılınç</t>
+          <t>Dr. Test05</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -531,7 +531,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dr. Sedef Özdemir</t>
+          <t>Dr. Test06</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -549,7 +549,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Dr. Ali Bulut</t>
+          <t>Dr. Test07</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -567,7 +567,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dr. Ayten Değirmencioğlu</t>
+          <t>Dr. Test08</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -585,7 +585,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dr. Merve Celep</t>
+          <t>Dr. Test09</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -603,7 +603,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dr. Orhan Güney</t>
+          <t>Dr. Test10</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -621,7 +621,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dr. Yusuf Emir Kumkumoğlu</t>
+          <t>Dr. Test11</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -639,7 +639,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dr. Mehmet Kamil Göktaş</t>
+          <t>Dr. Test12</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -657,7 +657,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dr. Kübra Yaşar</t>
+          <t>Dr. Test13</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -675,7 +675,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Dr. Muhammed Ali Yılmaz</t>
+          <t>Dr. Test14</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -693,7 +693,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dr. Türkü Berivan Karahan Ayvaz</t>
+          <t>Dr. Test15</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -711,7 +711,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dr. Evrim Zülal Aşlar</t>
+          <t>Dr. Test16</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -729,7 +729,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dr. Ayhan Çendik</t>
+          <t>Dr. Test17</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -747,7 +747,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dr. Belgin Aslan</t>
+          <t>Dr. Test18</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -765,7 +765,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dr. Kübra Tutal Şahin</t>
+          <t>Dr. Test19</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -783,7 +783,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dr. Tuğçe Eren</t>
+          <t>Dr. Test20</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -801,7 +801,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dr. İpek Durğun</t>
+          <t>Dr. Test21</t>
         </is>
       </c>
       <c r="B22" t="n">

</xml_diff>